<commit_message>
Update insights and wardrobe stats
</commit_message>
<xml_diff>
--- a/public/templates/wardrobe-import-template.xlsx
+++ b/public/templates/wardrobe-import-template.xlsx
@@ -31,7 +31,7 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="005C3B1E"/>
+      <color rgb="003D2B1F"/>
     </font>
   </fonts>
   <fills count="3">
@@ -43,7 +43,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F5EBDD"/>
+        <fgColor rgb="00EEDBC9"/>
       </patternFill>
     </fill>
   </fills>
@@ -429,33 +429,35 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X3"/>
+  <dimension ref="A1:Z3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
-    <col width="10" customWidth="1" min="10" max="10"/>
-    <col width="10" customWidth="1" min="11" max="11"/>
-    <col width="10" customWidth="1" min="12" max="12"/>
-    <col width="10" customWidth="1" min="13" max="13"/>
-    <col width="10" customWidth="1" min="14" max="14"/>
-    <col width="10" customWidth="1" min="15" max="15"/>
-    <col width="10" customWidth="1" min="16" max="16"/>
-    <col width="13" customWidth="1" min="17" max="17"/>
-    <col width="10" customWidth="1" min="18" max="18"/>
-    <col width="10" customWidth="1" min="19" max="19"/>
-    <col width="10" customWidth="1" min="20" max="20"/>
-    <col width="10" customWidth="1" min="21" max="21"/>
-    <col width="10" customWidth="1" min="22" max="22"/>
-    <col width="10" customWidth="1" min="23" max="23"/>
-    <col width="10" customWidth="1" min="24" max="24"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+    <col width="14" customWidth="1" min="16" max="16"/>
+    <col width="14" customWidth="1" min="17" max="17"/>
+    <col width="14" customWidth="1" min="18" max="18"/>
+    <col width="14" customWidth="1" min="19" max="19"/>
+    <col width="14" customWidth="1" min="20" max="20"/>
+    <col width="14" customWidth="1" min="21" max="21"/>
+    <col width="14" customWidth="1" min="22" max="22"/>
+    <col width="14" customWidth="1" min="23" max="23"/>
+    <col width="14" customWidth="1" min="24" max="24"/>
+    <col width="14" customWidth="1" min="25" max="25"/>
+    <col width="14" customWidth="1" min="26" max="26"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -486,114 +488,124 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>款式</t>
+          <t>颜色</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>颜色</t>
+          <t>设计元素</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>设计元素</t>
+          <t>材质</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>材质</t>
+          <t>袖型</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>袖型</t>
+          <t>领型</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>领型</t>
+          <t>宽松度</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>宽松度</t>
+          <t>廓形</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>廓形</t>
+          <t>风格</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>风格</t>
+          <t>季节</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>季节</t>
+          <t>价格</t>
         </is>
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
-          <t>价格</t>
+          <t>价格段</t>
         </is>
       </c>
       <c r="Q1" s="1" t="inlineStr">
         <is>
-          <t>价格段</t>
+          <t>穿着天数</t>
         </is>
       </c>
       <c r="R1" s="1" t="inlineStr">
         <is>
-          <t>穿着天数</t>
+          <t>单次价格</t>
         </is>
       </c>
       <c r="S1" s="1" t="inlineStr">
         <is>
-          <t>单次价格</t>
+          <t>购入年份</t>
         </is>
       </c>
       <c r="T1" s="1" t="inlineStr">
         <is>
-          <t>购入年份</t>
+          <t>购入月份</t>
         </is>
       </c>
       <c r="U1" s="1" t="inlineStr">
         <is>
+          <t>购入日期</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
           <t>购入渠道</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>衣服年龄</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>喜爱指数</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>标签</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>搭配</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>C001</t>
+          <t>CL001</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>c001.jpg</t>
+          <t>cl001.jpg</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Toteme</t>
+          <t>Mao by Mao</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -608,102 +620,108 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>衬衫</t>
+          <t>米色</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>白色</t>
+          <t>V领针织</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>落肩、口袋</t>
+          <t>羊毛</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>棉</t>
+          <t>长袖</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>长袖</t>
+          <t>V领</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>翻领</t>
+          <t>合身</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>宽松</t>
+          <t>直筒</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>直筒</t>
+          <t>通勤</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>极简</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>春季,秋季</t>
-        </is>
-      </c>
-      <c r="P2" t="n">
-        <v>1800</v>
-      </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>1000-3000</t>
-        </is>
+          <t>春/秋</t>
+        </is>
+      </c>
+      <c r="O2" t="n">
+        <v>699</v>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>500-1000</t>
+        </is>
+      </c>
+      <c r="Q2" t="n">
+        <v>12</v>
       </c>
       <c r="R2" t="n">
-        <v>8</v>
+        <v>58</v>
       </c>
       <c r="S2" t="n">
-        <v>225</v>
+        <v>2024</v>
       </c>
       <c r="T2" t="n">
-        <v>2024</v>
-      </c>
-      <c r="U2" t="inlineStr">
-        <is>
-          <t>连卡佛</t>
-        </is>
-      </c>
-      <c r="V2" t="n">
+        <v>9</v>
+      </c>
+      <c r="U2" t="n">
+        <v>18</v>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>线上精品店</t>
+        </is>
+      </c>
+      <c r="W2" t="n">
         <v>1</v>
       </c>
-      <c r="W2" t="n">
-        <v>9</v>
-      </c>
-      <c r="X2" t="inlineStr">
-        <is>
-          <t>通勤,极简</t>
+      <c r="X2" t="n">
+        <v>5</v>
+      </c>
+      <c r="Y2" t="inlineStr">
+        <is>
+          <t>通勤,基础款</t>
+        </is>
+      </c>
+      <c r="Z2" t="inlineStr">
+        <is>
+          <t>可配半裙</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>C002</t>
+          <t>CL002</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>c002.jpg</t>
+          <t>cl002.jpg</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>The Row</t>
+          <t>COS</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -713,82 +731,96 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>下装</t>
+          <t>外套</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>半裙</t>
+          <t>黑色</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>黑色</t>
+          <t>双排扣大衣</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>高腰、开衩</t>
+          <t>羊毛</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>羊毛</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
+          <t>长袖</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>翻领</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>宽松</t>
+        </is>
+      </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>合身</t>
+          <t>H型</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>A字</t>
+          <t>正式商务</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>通勤</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>秋季,冬季</t>
-        </is>
-      </c>
-      <c r="P3" t="n">
-        <v>3200</v>
-      </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>3000-5000</t>
-        </is>
+          <t>冬</t>
+        </is>
+      </c>
+      <c r="O3" t="n">
+        <v>2390</v>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>2000+</t>
+        </is>
+      </c>
+      <c r="Q3" t="n">
+        <v>8</v>
       </c>
       <c r="R3" t="n">
+        <v>299</v>
+      </c>
+      <c r="S3" t="n">
+        <v>2023</v>
+      </c>
+      <c r="T3" t="n">
+        <v>11</v>
+      </c>
+      <c r="U3" t="n">
         <v>6</v>
       </c>
-      <c r="S3" t="n">
-        <v>533</v>
-      </c>
-      <c r="T3" t="n">
-        <v>2023</v>
-      </c>
-      <c r="U3" t="inlineStr">
-        <is>
-          <t>品牌官网</t>
-        </is>
-      </c>
-      <c r="V3" t="n">
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>线下门店</t>
+        </is>
+      </c>
+      <c r="W3" t="n">
         <v>2</v>
       </c>
-      <c r="W3" t="n">
-        <v>10</v>
-      </c>
-      <c r="X3" t="inlineStr">
-        <is>
-          <t>通勤,正式</t>
+      <c r="X3" t="n">
+        <v>4</v>
+      </c>
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>正式,秋冬</t>
+        </is>
+      </c>
+      <c r="Z3" t="inlineStr">
+        <is>
+          <t>可配西裤</t>
         </is>
       </c>
     </row>
@@ -803,25 +835,26 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P3"/>
+  <dimension ref="A1:Q3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
-    <col width="10" customWidth="1" min="10" max="10"/>
-    <col width="13" customWidth="1" min="11" max="11"/>
-    <col width="10" customWidth="1" min="12" max="12"/>
-    <col width="10" customWidth="1" min="13" max="13"/>
-    <col width="10" customWidth="1" min="14" max="14"/>
-    <col width="10" customWidth="1" min="15" max="15"/>
-    <col width="10" customWidth="1" min="16" max="16"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="16.4" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+    <col width="14" customWidth="1" min="16" max="16"/>
+    <col width="14" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -852,55 +885,60 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>款式</t>
+          <t>颜色</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>颜色</t>
+          <t>设计元素</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>设计元素</t>
+          <t>季节</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>季节</t>
+          <t>价格</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>价格</t>
+          <t>价格段</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>价格段</t>
+          <t>穿着天数</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>穿着天数</t>
+          <t>单次价格</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>单次价格</t>
+          <t>购入年份</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>购入年份</t>
+          <t>购入月份</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
+          <t>购入日期</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
           <t>购入渠道</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>喜爱指数</t>
         </is>
@@ -909,17 +947,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>A001</t>
+          <t>AC001</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>a001.jpg</t>
+          <t>ac001.jpg</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Toteme</t>
+          <t>Acne Studios</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -929,69 +967,70 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>帽饰</t>
+          <t>围巾</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>棒球帽</t>
+          <t>灰色</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>藏蓝</t>
+          <t>流苏</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>刺绣logo</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>春季,夏季</t>
-        </is>
-      </c>
-      <c r="J2" t="n">
-        <v>680</v>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>500-1000</t>
-        </is>
+          <t>秋/冬</t>
+        </is>
+      </c>
+      <c r="I2" t="n">
+        <v>1200</v>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>1000-2000</t>
+        </is>
+      </c>
+      <c r="K2" t="n">
+        <v>20</v>
       </c>
       <c r="L2" t="n">
-        <v>12</v>
+        <v>60</v>
       </c>
       <c r="M2" t="n">
-        <v>57</v>
+        <v>2022</v>
       </c>
       <c r="N2" t="n">
-        <v>2024</v>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>品牌官网</t>
-        </is>
-      </c>
-      <c r="P2" t="n">
+        <v>10</v>
+      </c>
+      <c r="O2" t="n">
         <v>8</v>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>海外电商</t>
+        </is>
+      </c>
+      <c r="Q2" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>A002</t>
+          <t>AC002</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>a002.jpg</t>
+          <t>ac002.jpg</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Loro Piana</t>
+          <t>Celine</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -1001,53 +1040,54 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>围巾</t>
+          <t>眼镜</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>羊绒围巾</t>
+          <t>黑色</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>驼色</t>
+          <t>方框</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>流苏</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>秋季,冬季</t>
-        </is>
-      </c>
-      <c r="J3" t="n">
-        <v>2600</v>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>1000-3000</t>
-        </is>
+          <t>四季</t>
+        </is>
+      </c>
+      <c r="I3" t="n">
+        <v>3200</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>2000+</t>
+        </is>
+      </c>
+      <c r="K3" t="n">
+        <v>45</v>
       </c>
       <c r="L3" t="n">
-        <v>15</v>
+        <v>71</v>
       </c>
       <c r="M3" t="n">
-        <v>173</v>
+        <v>2021</v>
       </c>
       <c r="N3" t="n">
-        <v>2022</v>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>门店</t>
-        </is>
-      </c>
-      <c r="P3" t="n">
-        <v>9</v>
+        <v>5</v>
+      </c>
+      <c r="O3" t="n">
+        <v>14</v>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>线下门店</t>
+        </is>
+      </c>
+      <c r="Q3" t="n">
+        <v>4</v>
       </c>
     </row>
   </sheetData>
@@ -1061,27 +1101,29 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R3"/>
+  <dimension ref="A1:T3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
-    <col width="10" customWidth="1" min="10" max="10"/>
-    <col width="10" customWidth="1" min="11" max="11"/>
-    <col width="10" customWidth="1" min="12" max="12"/>
-    <col width="10" customWidth="1" min="13" max="13"/>
-    <col width="10" customWidth="1" min="14" max="14"/>
-    <col width="10" customWidth="1" min="15" max="15"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
     <col width="14" customWidth="1" min="16" max="16"/>
-    <col width="10" customWidth="1" min="17" max="17"/>
-    <col width="10" customWidth="1" min="18" max="18"/>
+    <col width="14" customWidth="1" min="17" max="17"/>
+    <col width="14" customWidth="1" min="18" max="18"/>
+    <col width="14" customWidth="1" min="19" max="19"/>
+    <col width="14" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1107,7 +1149,7 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>款式</t>
+          <t>类型</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
@@ -1162,15 +1204,25 @@
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
-          <t>购买时间</t>
+          <t>购入年份</t>
         </is>
       </c>
       <c r="Q1" s="1" t="inlineStr">
         <is>
+          <t>购入月份</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>购入日期</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
           <t>购买渠道</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>喜爱指数</t>
         </is>
@@ -1179,17 +1231,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>B001</t>
+          <t>BG001</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>b001.jpg</t>
+          <t>bg001.jpg</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Celine</t>
+          <t>Longchamp</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -1209,17 +1261,17 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>大号</t>
+          <t>中号</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>皮革</t>
+          <t>尼龙</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>金属扣</t>
+          <t>皮革提手</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -1229,51 +1281,55 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>通勤</t>
+          <t>职场通勤</t>
         </is>
       </c>
       <c r="L2" t="n">
-        <v>18500</v>
+        <v>980</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>10000+</t>
+          <t>500-1000</t>
         </is>
       </c>
       <c r="N2" t="n">
-        <v>40</v>
+        <v>120</v>
       </c>
       <c r="O2" t="n">
-        <v>463</v>
-      </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>2024-03-10</t>
-        </is>
-      </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>门店</t>
-        </is>
+        <v>8</v>
+      </c>
+      <c r="P2" t="n">
+        <v>2020</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>3</v>
       </c>
       <c r="R2" t="n">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>海外电商</t>
+        </is>
+      </c>
+      <c r="T2" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>B002</t>
+          <t>BG002</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>b002.jpg</t>
+          <t>bg002.jpg</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Loewe</t>
+          <t>The Row</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -1283,7 +1339,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>斜挎包</t>
+          <t>单肩包</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -1293,7 +1349,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>中号</t>
+          <t>小号</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -1303,45 +1359,49 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>拼接、压纹</t>
+          <t>极简廓形</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>秋季,冬季</t>
+          <t>秋/冬</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>出行</t>
+          <t>精致约会</t>
         </is>
       </c>
       <c r="L3" t="n">
-        <v>13800</v>
+        <v>15800</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>10000+</t>
+          <t>2000+</t>
         </is>
       </c>
       <c r="N3" t="n">
+        <v>18</v>
+      </c>
+      <c r="O3" t="n">
+        <v>878</v>
+      </c>
+      <c r="P3" t="n">
+        <v>2024</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>1</v>
+      </c>
+      <c r="R3" t="n">
         <v>22</v>
       </c>
-      <c r="O3" t="n">
-        <v>627</v>
-      </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>2023-11-02</t>
-        </is>
-      </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>品牌官网</t>
-        </is>
-      </c>
-      <c r="R3" t="n">
-        <v>8</v>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>线下门店</t>
+        </is>
+      </c>
+      <c r="T3" t="n">
+        <v>4</v>
       </c>
     </row>
   </sheetData>
@@ -1355,26 +1415,27 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q3"/>
+  <dimension ref="A1:R3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
-    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
     <col width="14" customWidth="1" min="11" max="11"/>
-    <col width="10" customWidth="1" min="12" max="12"/>
-    <col width="10" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
     <col width="14" customWidth="1" min="14" max="14"/>
-    <col width="10" customWidth="1" min="15" max="15"/>
-    <col width="10" customWidth="1" min="16" max="16"/>
-    <col width="10" customWidth="1" min="17" max="17"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+    <col width="14" customWidth="1" min="16" max="16"/>
+    <col width="14" customWidth="1" min="17" max="17"/>
+    <col width="14" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1400,7 +1461,7 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>款式</t>
+          <t>类型</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
@@ -1445,39 +1506,44 @@
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>购买时间</t>
+          <t>购入年份</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
+          <t>购入月份</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>购入日期</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
           <t>购买渠道</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>喜爱指数</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>现状</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>S001</t>
+          <t>SH001</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>s001.jpg</t>
+          <t>sh001.jpg</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>The Row</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -1487,76 +1553,75 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>乐福鞋</t>
+          <t>运动鞋</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>黑色</t>
+          <t>白色</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>方头</t>
+          <t>复古跑鞋</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>通勤</t>
+          <t>运动</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>春季,秋季</t>
+          <t>春/夏</t>
         </is>
       </c>
       <c r="J2" t="n">
-        <v>7200</v>
+        <v>899</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>5000-10000</t>
+          <t>500-1000</t>
         </is>
       </c>
       <c r="L2" t="n">
-        <v>18</v>
+        <v>55</v>
       </c>
       <c r="M2" t="n">
-        <v>400</v>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>2024-02-18</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>品牌官网</t>
-        </is>
+        <v>16</v>
+      </c>
+      <c r="N2" t="n">
+        <v>2024</v>
+      </c>
+      <c r="O2" t="n">
+        <v>4</v>
       </c>
       <c r="P2" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>常穿</t>
-        </is>
+          <t>线上旗舰店</t>
+        </is>
+      </c>
+      <c r="R2" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>S002</t>
+          <t>SH002</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>s002.jpg</t>
+          <t>sh002.jpg</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>New Balance</t>
+          <t>Church's</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -1566,60 +1631,59 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>运动鞋</t>
+          <t>乐福鞋</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>灰色</t>
+          <t>棕色</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>网面、拼色</t>
+          <t>厚底</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>日常</t>
+          <t>正式商务</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>四季</t>
+          <t>秋</t>
         </is>
       </c>
       <c r="J3" t="n">
-        <v>1299</v>
+        <v>5600</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>1000-3000</t>
+          <t>2000+</t>
         </is>
       </c>
       <c r="L3" t="n">
-        <v>35</v>
+        <v>22</v>
       </c>
       <c r="M3" t="n">
-        <v>37</v>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>2023-08-15</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>旗舰店</t>
-        </is>
+        <v>255</v>
+      </c>
+      <c r="N3" t="n">
+        <v>2023</v>
+      </c>
+      <c r="O3" t="n">
+        <v>9</v>
       </c>
       <c r="P3" t="n">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>常穿</t>
-        </is>
+          <t>线下门店</t>
+        </is>
+      </c>
+      <c r="R3" t="n">
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -1633,23 +1697,25 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N3"/>
+  <dimension ref="A1:P3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="17.6" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="10" customWidth="1" min="10" max="10"/>
-    <col width="10" customWidth="1" min="11" max="11"/>
-    <col width="10" customWidth="1" min="12" max="12"/>
-    <col width="10" customWidth="1" min="13" max="13"/>
-    <col width="10" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+    <col width="14" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1675,7 +1741,7 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>款式</t>
+          <t>类型</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
@@ -1715,10 +1781,20 @@
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
+          <t>购入月份</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>购入日期</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
           <t>渠道</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>喜爱指数</t>
         </is>
@@ -1727,12 +1803,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>J001</t>
+          <t>JW001</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>j001.jpg</t>
+          <t>jw001.jpg</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -1747,7 +1823,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>戒指</t>
+          <t>项链</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -1757,49 +1833,55 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>窄版素圈</t>
+          <t>经典圆环</t>
         </is>
       </c>
       <c r="H2" t="n">
-        <v>9800</v>
+        <v>18800</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>5000-10000</t>
+          <t>2000+</t>
         </is>
       </c>
       <c r="J2" t="n">
-        <v>28</v>
+        <v>36</v>
       </c>
       <c r="K2" t="n">
-        <v>350</v>
+        <v>522</v>
       </c>
       <c r="L2" t="n">
-        <v>2022</v>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>门店</t>
-        </is>
+        <v>2021</v>
+      </c>
+      <c r="M2" t="n">
+        <v>12</v>
       </c>
       <c r="N2" t="n">
-        <v>10</v>
+        <v>5</v>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>线下门店</t>
+        </is>
+      </c>
+      <c r="P2" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>J002</t>
+          <t>JW002</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>j002.jpg</t>
+          <t>jw002.jpg</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Van Cleef &amp; Arpels</t>
+          <t>Tiffany &amp; Co.</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -1809,43 +1891,49 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>项链</t>
+          <t>耳饰</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>金色</t>
+          <t>银色</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>四叶草</t>
+          <t>珍珠耳钉</t>
         </is>
       </c>
       <c r="H3" t="n">
-        <v>21500</v>
+        <v>6200</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>10000+</t>
+          <t>2000+</t>
         </is>
       </c>
       <c r="J3" t="n">
-        <v>16</v>
+        <v>28</v>
       </c>
       <c r="K3" t="n">
-        <v>1344</v>
+        <v>221</v>
       </c>
       <c r="L3" t="n">
-        <v>2023</v>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>门店</t>
-        </is>
+        <v>2022</v>
+      </c>
+      <c r="M3" t="n">
+        <v>6</v>
       </c>
       <c r="N3" t="n">
-        <v>9</v>
+        <v>20</v>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>海外电商</t>
+        </is>
+      </c>
+      <c r="P3" t="n">
+        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>